<commit_message>
Added dataa Enough data to begin plotting it on the night sky.
</commit_message>
<xml_diff>
--- a/SleepTimes.xlsx
+++ b/SleepTimes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UniWork\Creative Coding Dear Data Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56056D6F-5ECD-4783-8009-01C8F3D66C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95416588-7601-445B-8065-718D86604721}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EAC68948-DFEA-4671-8075-6E14F60634DA}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Data" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -60,10 +59,10 @@
     <t>Bed2</t>
   </si>
   <si>
-    <t>Sleep3</t>
+    <t>Date</t>
   </si>
   <si>
-    <t>Date</t>
+    <t>Sleep2</t>
   </si>
 </sst>
 </file>
@@ -524,7 +523,7 @@
     <tableColumn id="4" xr3:uid="{85B968B3-9D0E-448C-AC51-ADC52D581EFA}" name="Bed2" dataDxfId="2">
       <calculatedColumnFormula>B6*24</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{815EDEA4-75A9-4C6F-8361-30821BDAC15C}" name="Sleep3" dataDxfId="1">
+    <tableColumn id="5" xr3:uid="{815EDEA4-75A9-4C6F-8361-30821BDAC15C}" name="Sleep2" dataDxfId="1">
       <calculatedColumnFormula>C6*24</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{BC1C5660-F08A-4376-A0CD-AE5BAB6D1994}" name="Difference" dataDxfId="0">
@@ -873,7 +872,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="14" t="s">
         <v>2</v>
@@ -885,7 +884,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F5" s="11" t="s">
         <v>4</v>
@@ -1148,57 +1147,69 @@
       <c r="A17" s="6">
         <v>46318</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
+      <c r="B17" s="13">
+        <v>0.97777777777777775</v>
+      </c>
+      <c r="C17" s="13">
+        <v>1.0229166666666667</v>
+      </c>
       <c r="D17" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>23.466666666666665</v>
       </c>
       <c r="E17" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>24.55</v>
       </c>
       <c r="F17" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.0833333333333357</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="6">
         <v>46319</v>
       </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
+      <c r="B18" s="12">
+        <v>0.96805555555555556</v>
+      </c>
+      <c r="C18" s="12">
+        <v>5.7638888888888892E-2</v>
+      </c>
       <c r="D18" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>23.233333333333334</v>
       </c>
       <c r="E18" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.3833333333333333</v>
       </c>
       <c r="F18" s="7">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2.1499999999999986</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>46320</v>
       </c>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
+      <c r="B19" s="13">
+        <v>0.89722222222222225</v>
+      </c>
+      <c r="C19" s="13">
+        <v>0.94652777777777775</v>
+      </c>
       <c r="D19" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>21.533333333333335</v>
       </c>
       <c r="E19" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>22.716666666666665</v>
       </c>
       <c r="F19" s="8">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1.18333333333333</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>